<commit_message>
edits from JB. Revert plots to end in 2023 to match assessment data
</commit_message>
<xml_diff>
--- a/docs/table_template.xlsx
+++ b/docs/table_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\stephanie.owen\Documents\longfinESP\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07CB7612-1A22-455A-BB06-14A2A5EE9D11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EB3FCC3-B51A-4746-87DA-24153E70766C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,14 +28,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="25">
   <si>
     <t>Indicator (units)</t>
   </si>
   <si>
-    <t>Status in 2024</t>
-  </si>
-  <si>
     <t>Implications</t>
   </si>
   <si>
@@ -48,63 +45,69 @@
     <t>h</t>
   </si>
   <si>
-    <t xml:space="preserve">Commercial landings (millions of lbs.)
+    <t>Western Gulf Stream Index (shift in the western part of the Gulf Stream North wall: mean position: &gt;0 = more northerly, &lt;0 = more southerly)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Environmental dynamics vary between locations/timing of the summer and winter squid fisheries. An increase in landings since 2020 but decrease in number of vessels could indicate targeted trips in specific times of year and fishers targeting other species when longfin are not available. </t>
+  </si>
+  <si>
+    <t>Number of commercial vessels (#  of federally-permitted vessels landing over 1lb of longfin squid)</t>
+  </si>
+  <si>
+    <t>Inshore temperature thresholds (around 14°C) initiate migration of squid from offshore overwintering habitats. Longfin squid seasonal distribution and growth rates are likely temperature dependent, avoiding water &lt;8°C. Stronger and/or more persistent Mid-Atlantic Cold Pool conditions (not shown) may limit habitat availability (https://noaa-edab.github.io/catalog/cold_pool.html).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Since the mid-1990s, north and westward shifts in the Gulf Stream have resulted in an increase in warm core rings and deep water, high salinity heat waves. The position of the Gulf Stream influences seasonal temperature and water mass mixing dynamics that affect longfin squid habitat suitability, temperature-dependent growth, and prey availability (https://noaa-edab.github.io/catalog/gsi.html). </t>
+  </si>
+  <si>
+    <t>Commercial revenue (millions, inflation adjusted to 2025 USD)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Commercial landings (millions of lbs)
 </t>
   </si>
   <si>
-    <t>Western Gulf Stream Index (shift in the western part of the Gulf Stream North wall: mean position: &gt;0 = more northerly, &lt;0 = more southerly)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bottom temperature in MAB and SNE(°C) </t>
-  </si>
-  <si>
-    <t>BottomT_2025-04-17.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Environmental dynamics vary between locations/timing of the summer and winter squid fisheries. An increase in landings since 2020 but decrease in number of vessels could indicate targeted trips in specific times of year and fishers targeting other species when longfin are not available. </t>
-  </si>
-  <si>
-    <t>Number of commercial vessels (#  of federally-permitted vessels landing over 1lb of longfin squid)</t>
-  </si>
-  <si>
-    <t>Inshore temperature thresholds (around 14°C) initiate migration of squid from offshore overwintering habitats. Longfin squid seasonal distribution and growth rates are likely temperature dependent, avoiding water &lt;8°C. Stronger and/or more persistent Mid-Atlantic Cold Pool conditions (not shown) may limit habitat availability (https://noaa-edab.github.io/catalog/cold_pool.html).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Since the mid-1990s, north and westward shifts in the Gulf Stream have resulted in an increase in warm core rings and deep water, high salinity heat waves. The position of the Gulf Stream influences seasonal temperature and water mass mixing dynamics that affect longfin squid habitat suitability, temperature-dependent growth, and prey availability (https://noaa-edab.github.io/catalog/gsi.html). </t>
-  </si>
-  <si>
-    <t>Above long term (1996-2024) average (Fall); near long term (1996-2024) average (Spring)</t>
-  </si>
-  <si>
-    <t>Near long term (1996-2025) average</t>
-  </si>
-  <si>
-    <t>western gulf stream index_2026-02-23.png</t>
-  </si>
-  <si>
-    <t>Below long term (1996-2025) average</t>
+    <t>Status in 2023</t>
+  </si>
+  <si>
+    <t>Near long term (1996-2023) average</t>
+  </si>
+  <si>
+    <t>Below long term (1996-2023) average</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bottom temperature in Mid-Atlantic Bight (MAB) and Southern New England (SNE)(°C) </t>
+  </si>
+  <si>
+    <t>BottomT_2026-06-08.png</t>
+  </si>
+  <si>
+    <t>Near long term (1996-2023) average (Fall and Spring)</t>
+  </si>
+  <si>
+    <t>western gulf stream index_2026-06-08.png</t>
+  </si>
+  <si>
+    <t>Above long term (1996-2023) average</t>
+  </si>
+  <si>
+    <t>Commercial_LONGFINSQUID_Landings_LBS_2026-06-08.png</t>
+  </si>
+  <si>
+    <t>N_Commercial_Vessels_Landing_LONGFINSQUID_2026-06-08.png</t>
+  </si>
+  <si>
+    <t>TOTALANNUALREV_LONGFINSQUID_2025Dols_2026-06-08.png</t>
   </si>
   <si>
     <t xml:space="preserve">Number of commercial vessels has been steadily
-decreasing since around 2000 (although has slightly increased in 2025) consistent with
+decreasing since around 2000  consistent with
 decreasing fleet diversity and continued risk to
 fishery resilience [7]. Permit requalification in 2019 and a decrease in the post-closure trip  limit for trimester 2 may cap participation, although these actions were designed to accommodate recent fishing trends and activity. </t>
   </si>
   <si>
-    <t>Commercial revenue (millions, inflation adjusted to 2025 USD)</t>
-  </si>
-  <si>
-    <t>Average longfin ex-vessel prices in 2024 increased slightly from 2023 (+10%). Commercial revenue has decreased since 2022, driven by the overall
+    <t>Commercial revenue has decreased since 2022, driven by the overall
 decrease in landings by 23% [7].</t>
-  </si>
-  <si>
-    <t>Commercial_LONGFINSQUID_Landings_LBS_2026-02-25.png</t>
-  </si>
-  <si>
-    <t>N_Commercial_Vessels_Landing_LONGFINSQUID_2026-02-25.png</t>
-  </si>
-  <si>
-    <t>TOTALANNUALREV_LONGFINSQUID_2025Dols_2026-02-25.png</t>
   </si>
 </sst>
 </file>
@@ -523,33 +526,33 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="F1" s="4" t="s">
         <v>4</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>10</v>
-      </c>
       <c r="D2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E2">
         <v>3</v>
@@ -558,18 +561,18 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="185.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" ht="172.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="B3" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="D3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E3">
         <v>3</v>
@@ -578,18 +581,18 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="79.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" ht="40.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="4" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="B4" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="D4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E4">
         <v>3</v>
@@ -600,16 +603,16 @@
     </row>
     <row r="5" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B5" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="D5" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E5">
         <v>3</v>
@@ -620,16 +623,16 @@
     </row>
     <row r="6" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B6" t="s">
-        <v>14</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="D6" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="E6">
         <v>3</v>

</xml_diff>